<commit_message>
fix(telemetry): base device last-seen on the receive clock so skewed clocks can't fake silence (F-J1/F-J3)
resolve_last_telemetry_at returned the received_at of the row with the
largest device recorded_at, so one reading stamped in the future stayed
'latest' and every newer arrival looked like silence (false device-offline
alerts) - the opposite of what its docstring promised. It now takes the
newest received_at, served by a new (vehicle_id, received_at DESC) index on
the hypertable (model, baseline migration, DBML, regenerated views).

Integration test proves it (fails on the old logic); make db-check clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/01-requirements/domain-model/domain-model.xlsx
+++ b/docs/01-requirements/domain-model/domain-model.xlsx
@@ -3692,7 +3692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4589,16 +4589,16 @@
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
     </row>
-    <row r="33" ht="27" customHeight="1">
+    <row r="33" ht="108" customHeight="1">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>ix_vehicle_telemetry_message_uuid</t>
+          <t>ix_vehicle_telemetry_vehicle_received</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>message_uuid</t>
+          <t>vehicle_id, received_at DESC</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -4607,27 +4607,51 @@
         </is>
       </c>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Last time the backend heard from a vehicle (F-J1/F-J3 device-health monitor); uses the receive clock, which a skewed device clock cannot move. @vi Lần cuối backend nhận dữ liệu từ xe (giám sát thiết bị F-J1/F-J3); dùng đồng hồ nhận của backend, không bị lệch giờ thiết bị làm sai.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="27" customHeight="1">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>uq_telematic_recorded_at</t>
+          <t>ix_vehicle_telemetry_message_uuid</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>telematic_id, recorded_at</t>
+          <t>message_uuid</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>có</t>
+          <t>không</t>
         </is>
       </c>
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="27" customHeight="1">
+      <c r="A35" s="6" t="n"/>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>uq_telematic_recorded_at</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>telematic_id, recorded_at</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A6:H29"/>

</xml_diff>

<commit_message>
feat(db): schema and settings for the happy-path completion round (phase A)
- telematics: full unique constraint on vehicle_id -> partial unique index
  uq_telematics_active_vehicle (WHERE deleted_at IS NULL), so a
  soft-deleted device no longer blocks a replacement (future.md #82)
- notificationtype: SOS_ALERT (F-I2), GEOFENCE_ALERT (F-A5)
- geofences table (fleet domain; account_id stays planned until customer
  accounts exist)
- settings: TELEMETRY_ONLINE_THRESHOLD_SECONDS, TELEMETRY_ENERGY_COST_PER_
  KWH_VND, TELEMETRY_SOH_ALERT_THRESHOLD_PERCENT, TELEMETRY_BATTERY_HEALTH_
  MAX_RANGE_DAYS, APP_REPORT_TIMEZONE, CHARGING_ENERGY_SERIES_MAX_RANGE_DAYS;
  TELEMETRY_REPORT_MAX_RANGE_DAYS 31 -> 366 for monthly breakdowns
- DBML (18 built tables) and views regenerated; planner
  backend-happy-path-completion.md with the 12 decisions taken

db-reset + db-check clean; integration 6/6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/01-requirements/domain-model/domain-model.xlsx
+++ b/docs/01-requirements/domain-model/domain-model.xlsx
@@ -15,14 +15,14 @@
     <sheet name="access_audit_logs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="vehicles" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="vehicle_ownerships" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="geofences" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="telematics" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="vehicle_telemetry" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="drivers" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="driver_vehicle_assignments" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="charging_credentials" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="fleets" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="fleet_vehicle_memberships" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="telematics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="vehicle_telemetry" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="drivers" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="driver_vehicle_assignments" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="charging_credentials" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="fleets" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="fleet_vehicle_memberships" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="geofences" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="charging_stations" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="charging_evses" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="charging_connectors" sheetId="19" state="visible" r:id="rId19"/>
@@ -60,14 +60,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'access_audit_logs'!$A$6:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'vehicles'!$A$6:$H$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'vehicle_ownerships'!$A$6:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'geofences'!$A$6:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'telematics'!$A$6:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'vehicle_telemetry'!$A$6:$H$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'drivers'!$A$6:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'driver_vehicle_assignments'!$A$6:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'charging_credentials'!$A$6:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'fleets'!$A$6:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'fleet_vehicle_memberships'!$A$6:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'telematics'!$A$6:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'vehicle_telemetry'!$A$6:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'drivers'!$A$6:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'driver_vehicle_assignments'!$A$6:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'charging_credentials'!$A$6:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'fleets'!$A$6:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'fleet_vehicle_memberships'!$A$6:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'geofences'!$A$6:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'charging_stations'!$A$6:$H$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'charging_evses'!$A$6:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'charging_connectors'!$A$6:$H$17</definedName>
@@ -885,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="67.5" customHeight="1">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Xe (vehicles)</t>
@@ -893,7 +893,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>3 bảng</t>
+          <t>2 bảng</t>
         </is>
       </c>
       <c r="C12" s="5" t="n"/>
@@ -903,8 +903,7 @@
         <is>
           <t>Bản thân chiếc xe tải: định danh (VIN, biển số), thông số và trạng thái kích hoạt.
 • Tại mỗi thời điểm, một xe thuộc một tài khoản khách hàng (D1, D3).
-• Lịch sử sở hữu ghi lại mỗi lần đổi chủ, để dữ liệu cũ vẫn thuộc chủ cũ.
-• Khách hàng định nghĩa vùng địa lý (geofence) để nhận cảnh báo vị trí (F-A5).</t>
+• Lịch sử sở hữu ghi lại mỗi lần đổi chủ, để dữ liệu cũ vẫn thuộc chủ cũ.</t>
         </is>
       </c>
     </row>
@@ -988,61 +987,21 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Xe (vehicles)</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>geofences</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Vùng địa lý (geofence)</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Khách hàng</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>F-A5</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Một khu vực do khách hàng định nghĩa để cảnh báo khi xe vào/ra.</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>→ Mở</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="54" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Thiết bị telematics (telematics)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>1 bảng</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Các thiết bị telematics (T-box) gửi dữ liệu xe qua MQTT.
 • Một thiết bị gắn trên tối đa một xe, và một xe có tối đa một thiết bị.
@@ -1050,61 +1009,61 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="16" ht="27" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Thiết bị telematics (telematics)</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>telematics</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Thiết bị telematics</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Chưa quyết định</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>F-G1, F-J1, F-J2, F-J3</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Một thiết bị telematics và chiếc xe nó đang gắn. Thiết bị thuộc khách hàng hay G3 là quyết định D6.</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G16" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="67.5" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="17" ht="67.5" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Dữ liệu vận hành xe (telemetry)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>1 bảng</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Mọi thứ xe gửi về: vị trí, pin, động cơ, mã lỗi. Cảnh báo và báo cáo năng lượng được tính từ dữ liệu này.
 • Mỗi bản ghi đến từ một thiết bị và được lưu theo một xe.
@@ -1112,61 +1071,61 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="40.5" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="18" ht="40.5" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Dữ liệu vận hành xe (telemetry)</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>vehicle_telemetry</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Dữ liệu vận hành xe</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>F-A1, F-A2, F-A3, F-A4, F-A6, F-C6</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Một bản ghi dữ liệu xe gửi về, mỗi 5-10 giây một bản ghi cho mỗi xe: bảng lớn nhất hệ thống.</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G18" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>→ Mở</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="81" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="19" ht="81" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Tài xế (drivers)</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>3 bảng</t>
         </is>
       </c>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Những người lái xe và cách họ xác thực tại trụ sạc.
 • Một tài xế thuộc một tài khoản khách hàng (D1).
@@ -1175,6 +1134,46 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Tài xế (drivers)</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>drivers</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Tài xế</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Khách hàng</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>F-E4</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Một tài xế do khách hàng tuyển dụng (hoặc chính là khách hàng).</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>→ Mở</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
@@ -1183,12 +1182,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>drivers</t>
+          <t>driver_vehicle_assignments</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Tài xế</t>
+          <t>Phân công tài xế - xe</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1203,11 +1202,11 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Một tài xế do khách hàng tuyển dụng (hoặc chính là khách hàng).</t>
+          <t>Tài xế nào lái xe nào, trong khoảng thời gian nào (lịch sử mở/đóng).</t>
         </is>
       </c>
       <c r="G21" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
@@ -1215,7 +1214,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Tài xế (drivers)</t>
@@ -1223,12 +1222,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>driver_vehicle_assignments</t>
+          <t>charging_credentials</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Phân công tài xế - xe</t>
+          <t>Phương thức xác thực sạc</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1238,12 +1237,12 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>F-E4</t>
+          <t>F-B2, F-C6, F-H1</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Tài xế nào lái xe nào, trong khoảng thời gian nào (lịch sử mở/đóng).</t>
+          <t>Cách trụ sạc nhận biết ai đang sạc. Nối mã idTag thô của phiên sạc với tài xế và tài khoản. Việc đặt ở miền Tài xế là tạm thời.</t>
         </is>
       </c>
       <c r="G22" s="6" t="n">
@@ -1255,69 +1254,70 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Tài xế (drivers)</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>charging_credentials</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Phương thức xác thực sạc</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Khách hàng</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>F-B2, F-C6, F-H1</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Cách trụ sạc nhận biết ai đang sạc. Nối mã idTag thô của phiên sạc với tài xế và tài khoản. Việc đặt ở miền Tài xế là tạm thời.</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>→ Mở</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="54" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="23" ht="81" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Đội xe (fleet)</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>2 bảng</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>3 bảng</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Nhóm xe do một quản lý đội xe điều hành.
 • Một đội xe thuộc một tài khoản khách hàng (D1, D2).
-• Tại mỗi thời điểm, một xe thuộc tối đa một đội; một đội có nhiều xe. Thành viên đội lưu lại lịch sử.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="27" customHeight="1">
+• Tại mỗi thời điểm, một xe thuộc tối đa một đội; một đội có nhiều xe. Thành viên đội lưu lại lịch sử.
+• Vùng địa lý (geofence) của đội xe phát cảnh báo khi xe thành viên đi vào hoặc ra (F-A5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="27" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Đội xe (fleet)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>fleets</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Đội xe</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Khách hàng</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>F-E1</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Một nhóm xe có tên. Đội xe là chính khách hàng hay là nhóm con bên trong khách hàng là quyết định D2.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>→ Mở</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Đội xe (fleet)</t>
@@ -1325,12 +1325,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>fleets</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Đội xe</t>
+          <t>Thành viên đội xe</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Một nhóm xe có tên. Đội xe là chính khách hàng hay là nhóm con bên trong khách hàng là quyết định D2.</t>
+          <t>Xe nào thuộc đội nào, trong khoảng thời gian nào (lịch sử mở/đóng).</t>
         </is>
       </c>
       <c r="G25" s="6" t="n">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Đội xe (fleet)</t>
@@ -1365,12 +1365,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>fleet_vehicle_memberships</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Thành viên đội xe</t>
+          <t>Vùng địa lý (geofence)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1380,12 +1380,12 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>F-E1</t>
+          <t>F-A5</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Xe nào thuộc đội nào, trong khoảng thời gian nào (lịch sử mở/đóng).</t>
+          <t>Một khu vực mà khi xe thuộc đội xe đi vào hoặc ra sẽ phát cảnh báo. Gắn với đội xe cho đến khi có tài khoản khách hàng (sau đó chuyển sang tài khoản).</t>
         </is>
       </c>
       <c r="G26" s="6" t="n">
@@ -2997,30 +2997,30 @@
     <hyperlink ref="B14" location="'vehicle_ownerships'!A1"/>
     <hyperlink ref="C14" location="'vehicle_ownerships'!A1"/>
     <hyperlink ref="H14" location="'vehicle_ownerships'!A1"/>
-    <hyperlink ref="B15" location="'geofences'!A1"/>
-    <hyperlink ref="C15" location="'geofences'!A1"/>
-    <hyperlink ref="H15" location="'geofences'!A1"/>
-    <hyperlink ref="B17" location="'telematics'!A1"/>
-    <hyperlink ref="C17" location="'telematics'!A1"/>
-    <hyperlink ref="H17" location="'telematics'!A1"/>
-    <hyperlink ref="B19" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="C19" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="H19" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="B21" location="'drivers'!A1"/>
-    <hyperlink ref="C21" location="'drivers'!A1"/>
-    <hyperlink ref="H21" location="'drivers'!A1"/>
-    <hyperlink ref="B22" location="'driver_vehicle_assignments'!A1"/>
-    <hyperlink ref="C22" location="'driver_vehicle_assignments'!A1"/>
-    <hyperlink ref="H22" location="'driver_vehicle_assignments'!A1"/>
-    <hyperlink ref="B23" location="'charging_credentials'!A1"/>
-    <hyperlink ref="C23" location="'charging_credentials'!A1"/>
-    <hyperlink ref="H23" location="'charging_credentials'!A1"/>
-    <hyperlink ref="B25" location="'fleets'!A1"/>
-    <hyperlink ref="C25" location="'fleets'!A1"/>
-    <hyperlink ref="H25" location="'fleets'!A1"/>
-    <hyperlink ref="B26" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="C26" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="H26" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B16" location="'telematics'!A1"/>
+    <hyperlink ref="C16" location="'telematics'!A1"/>
+    <hyperlink ref="H16" location="'telematics'!A1"/>
+    <hyperlink ref="B18" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="C18" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="H18" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B20" location="'drivers'!A1"/>
+    <hyperlink ref="C20" location="'drivers'!A1"/>
+    <hyperlink ref="H20" location="'drivers'!A1"/>
+    <hyperlink ref="B21" location="'driver_vehicle_assignments'!A1"/>
+    <hyperlink ref="C21" location="'driver_vehicle_assignments'!A1"/>
+    <hyperlink ref="H21" location="'driver_vehicle_assignments'!A1"/>
+    <hyperlink ref="B22" location="'charging_credentials'!A1"/>
+    <hyperlink ref="C22" location="'charging_credentials'!A1"/>
+    <hyperlink ref="H22" location="'charging_credentials'!A1"/>
+    <hyperlink ref="B24" location="'fleets'!A1"/>
+    <hyperlink ref="C24" location="'fleets'!A1"/>
+    <hyperlink ref="H24" location="'fleets'!A1"/>
+    <hyperlink ref="B25" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="C25" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="H25" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B26" location="'geofences'!A1"/>
+    <hyperlink ref="C26" location="'geofences'!A1"/>
+    <hyperlink ref="H26" location="'geofences'!A1"/>
     <hyperlink ref="B28" location="'charging_stations'!A1"/>
     <hyperlink ref="C28" location="'charging_stations'!A1"/>
     <hyperlink ref="H28" location="'charging_stations'!A1"/>
@@ -3116,582 +3116,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>telematics: Thiết bị telematics</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>← Tổng quan</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Miền nghiệp vụ: Thiết bị telematics (telematics)   ·   Chủ sở hữu dữ liệu: Chưa quyết định   ·   Tính năng: F-G1, F-J1, F-J2, F-J3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Một thiết bị telematics và chiếc xe nó đang gắn. Thiết bị thuộc khách hàng hay G3 là quyết định D6.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Cho phép rỗng</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Khóa</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Tham chiếu tới</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Ý nghĩa</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Ví dụ</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>telematic_id</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Mã nội bộ của thiết bị telematics.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>2c8e5a1d-9f3b-4d7c-b2e6-8a1f0c5d9e55</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>telematic_serial</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>varchar(50)</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>UQ</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Số serial in trên thiết bị; cũng là định danh MQTT, duy nhất.</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>TBX-2409-000123</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FK UQ</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>vehicles.vehicle_id (khi xóa: đặt về NULL)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Xe mà thiết bị đang gắn; NULL khi đã tháo.</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>telematicstatus</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Trạng thái vận hành của thiết bị.</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>firmware_version</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>varchar(50)</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Phiên bản firmware đang chạy trên thiết bị.</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>1.4.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="27" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>telemetry_interval_seconds</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Chu kỳ gửi dữ liệu (giây) đã đẩy xuống thiết bị qua MQTT lần gần nhất (F-J2); NULL trước lần đẩy đầu tiên.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>config_pushed_at</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm đẩy chu kỳ đó lần gần nhất; NULL trước lần đẩy đầu tiên.</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-12T03:00:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm tạo bản ghi (UTC).</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01T02:00:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-10T07:15:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>deleted_at</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Thời điểm xóa mềm; NULL khi bản ghi còn hiệu lực. Không bao giờ xóa hẳn.</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Kiểu enum</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Giá trị cho phép</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>telematicstatus</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>ACTIVE, INACTIVE, MAINTENANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Chỉ mục (index)</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Các cột</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Duy nhất</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_status</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-    </row>
-    <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_telematic_serial</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>telematic_serial</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>có</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>ix_telematics_vehicle_id</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>vehicle_id</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Được tham chiếu bởi bảng</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Cột</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>vehicle_telemetry</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>telematic_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A6:H16"/>
-  <hyperlinks>
-    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F9" location="'vehicles'!A1"/>
-    <hyperlink ref="B27" location="'vehicle_telemetry'!A1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4665,7 +4089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5338,7 +4762,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5857,7 +5281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6266,13 +5690,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6747,14 +6171,27 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="27" customHeight="1">
+    <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="7" t="inlineStr">
         <is>
+          <t>geofences</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>fleet_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
           <t>charging_policy_assignments</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>fleet_id</t>
         </is>
@@ -6766,13 +6203,14 @@
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
     <hyperlink ref="F8" location="'customer_accounts'!A1"/>
     <hyperlink ref="B24" location="'fleet_vehicle_memberships'!A1"/>
-    <hyperlink ref="B25" location="'charging_policy_assignments'!A1"/>
+    <hyperlink ref="B25" location="'geofences'!A1"/>
+    <hyperlink ref="B26" location="'charging_policy_assignments'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7262,6 +6700,428 @@
     <hyperlink ref="F8" location="'customer_accounts'!A1"/>
     <hyperlink ref="F9" location="'fleets'!A1"/>
     <hyperlink ref="F10" location="'vehicles'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>geofences: Vùng địa lý (geofence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>← Tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Miền nghiệp vụ: Đội xe (fleet)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Một khu vực mà khi xe thuộc đội xe đi vào hoặc ra sẽ phát cảnh báo. Gắn với đội xe cho đến khi có tài khoản khách hàng (sau đó chuyển sang tài khoản).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu dữ liệu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cho phép rỗng</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Khóa</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tham chiếu tới</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>geofence_id</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Mã nội bộ của vùng địa lý.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>00000003-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="27" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>fleet_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>fleets.fleet_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Đội xe mà các xe thành viên hiện tại chịu áp dụng vùng này.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>8d5f2b7e-1a9c-4f3d-b8e2-6c0a4d9f1e77</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="27" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>customer_accounts.account_id (khi xóa: chặn xóa)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Tài khoản khách hàng đã tạo vùng, khi có tài khoản; trước đó vùng gắn với một đội xe. (xem quyết định D1)</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>varchar(100)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Tên hiển thị trong cảnh báo.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Kho Tân Uyên</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="27" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>boundary</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>geography(POLYGON,4326)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Ranh giới vùng, dạng đa giác WGS84 (kinh độ trước). Không có chỉ mục không gian: luôn lọc theo đội xe trước.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>POLYGON((106.70 11.05, 106.72 11.05, 106.72 11.07, 106.70 11.07, 106.70 11.05))</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm tạo bản ghi (UTC).</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-01T02:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="27" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm xóa mềm; NULL khi bản ghi còn hiệu lực. Không bao giờ xóa hẳn.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>ix_geofences_fleet_id</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>fleet_id</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:H14"/>
+  <hyperlinks>
+    <hyperlink ref="A2" location="'Tổng quan'!A1"/>
+    <hyperlink ref="F8" location="'fleets'!A1"/>
+    <hyperlink ref="F9" location="'customer_accounts'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9713,7 +9573,7 @@
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>geofences</t>
+          <t>vehicle_telemetry</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -9726,7 +9586,7 @@
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>vehicle_telemetry</t>
+          <t>drivers</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -9735,11 +9595,11 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>drivers</t>
+          <t>driver_vehicle_assignments</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -9748,11 +9608,11 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="27" customHeight="1">
+    <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>driver_vehicle_assignments</t>
+          <t>charging_credentials</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -9765,7 +9625,7 @@
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>charging_credentials</t>
+          <t>fleets</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -9774,11 +9634,11 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>fleets</t>
+          <t>fleet_vehicle_memberships</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -9787,11 +9647,11 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="27" customHeight="1">
+    <row r="28">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>fleet_vehicle_memberships</t>
+          <t>geofences</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -10004,13 +9864,13 @@
     <hyperlink ref="B19" location="'access_audit_logs'!A1"/>
     <hyperlink ref="B20" location="'vehicles'!A1"/>
     <hyperlink ref="B21" location="'vehicle_ownerships'!A1"/>
-    <hyperlink ref="B22" location="'geofences'!A1"/>
-    <hyperlink ref="B23" location="'vehicle_telemetry'!A1"/>
-    <hyperlink ref="B24" location="'drivers'!A1"/>
-    <hyperlink ref="B25" location="'driver_vehicle_assignments'!A1"/>
-    <hyperlink ref="B26" location="'charging_credentials'!A1"/>
-    <hyperlink ref="B27" location="'fleets'!A1"/>
-    <hyperlink ref="B28" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B22" location="'vehicle_telemetry'!A1"/>
+    <hyperlink ref="B23" location="'drivers'!A1"/>
+    <hyperlink ref="B24" location="'driver_vehicle_assignments'!A1"/>
+    <hyperlink ref="B25" location="'charging_credentials'!A1"/>
+    <hyperlink ref="B26" location="'fleets'!A1"/>
+    <hyperlink ref="B27" location="'fleet_vehicle_memberships'!A1"/>
+    <hyperlink ref="B28" location="'geofences'!A1"/>
     <hyperlink ref="B29" location="'charging_reservations'!A1"/>
     <hyperlink ref="B30" location="'charging_sessions'!A1"/>
     <hyperlink ref="B31" location="'notifications'!A1"/>
@@ -13474,7 +13334,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="54" customHeight="1">
+    <row r="19" ht="67.5" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="inlineStr">
         <is>
@@ -13483,7 +13343,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>BATTERY_ALERT, ANOMALY_ALERT, SOH_ALERT, DEVICE_OFFLINE_ALERT</t>
+          <t>BATTERY_ALERT, ANOMALY_ALERT, SOH_ALERT, DEVICE_OFFLINE_ALERT, SOS_ALERT, GEOFENCE_ALERT</t>
         </is>
       </c>
     </row>
@@ -23730,7 +23590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -23746,7 +23606,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>geofences: Vùng địa lý (geofence)</t>
+          <t>telematics: Thiết bị telematics</t>
         </is>
       </c>
     </row>
@@ -23760,14 +23620,14 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Miền nghiệp vụ: Xe (vehicles)   ·   Chủ sở hữu dữ liệu: Khách hàng   ·   Tính năng: F-A5</t>
+          <t>Miền nghiệp vụ: Thiết bị telematics (telematics)   ·   Chủ sở hữu dữ liệu: Chưa quyết định   ·   Tính năng: F-G1, F-J1, F-J2, F-J3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Một khu vực do khách hàng định nghĩa để cảnh báo khi xe vào/ra.</t>
+          <t>Một thiết bị telematics và chiếc xe nó đang gắn. Thiết bị thuộc khách hàng hay G3 là quyết định D6.</t>
         </is>
       </c>
     </row>
@@ -23820,7 +23680,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>geofence_id</t>
+          <t>telematic_id</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -23841,12 +23701,12 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Mã nội bộ của vùng địa lý.</t>
+          <t>Mã nội bộ của thiết bị telematics.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>00000003-5a6b-4c7d-8e9f-0a1b2c3d4e5f</t>
+          <t>2c8e5a1d-9f3b-4d7c-b2e6-8a1f0c5d9e55</t>
         </is>
       </c>
     </row>
@@ -23856,12 +23716,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>account_id</t>
+          <t>telematic_serial</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -23871,69 +23731,73 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>customer_accounts.account_id (khi xóa: chặn xóa)</t>
-        </is>
-      </c>
+          <t>UQ</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản khách hàng đã tạo vùng.</t>
+          <t>Số serial in trên thiết bị; cũng là định danh MQTT, duy nhất.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>3f6c2a1e-8b4d-4e2a-9c1f-0a7d5b2e4c11</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>TBX-2409-000123</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>vehicle_id</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>varchar(100)</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>không</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>vehicles.vehicle_id (khi xóa: đặt về NULL)</t>
+        </is>
+      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Tên hiển thị trong cảnh báo.</t>
+          <t>Xe mà thiết bị đang gắn; NULL khi đã tháo. Mỗi xe có tối đa một thiết bị còn hiệu lực (chưa xóa mềm).</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Kho Tân Uyên</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="27" customHeight="1">
+          <t>7a4c1e9b-3d2f-4b8a-a6c5-1e0d9f8b7a44</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>boundary</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>geography(Polygon,4326)</t>
+          <t>telematicstatus</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -23945,12 +23809,12 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Ranh giới vùng, dạng đa giác WGS84.</t>
+          <t>Trạng thái vận hành của thiết bị.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>POLYGON((106.70 11.05, 106.72 11.05, 106.72 11.07, 106.70 11.07, 106.70 11.05))</t>
+          <t>ACTIVE</t>
         </is>
       </c>
     </row>
@@ -23960,37 +23824,361 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>firmware_version</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>varchar(50)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>không</t>
+          <t>có</t>
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="inlineStr">
         <is>
+          <t>Phiên bản firmware đang chạy trên thiết bị.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>1.4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="27" customHeight="1">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>telemetry_interval_seconds</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Chu kỳ gửi dữ liệu (giây) đã đẩy xuống thiết bị qua MQTT lần gần nhất (F-J2); NULL trước lần đẩy đầu tiên.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="27" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>config_pushed_at</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm đẩy chu kỳ đó lần gần nhất; NULL trước lần đẩy đầu tiên.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-12T03:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
           <t>Thời điểm tạo bản ghi (UTC).</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>2026-09-01T02:00:00Z</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm bản ghi được sửa gần nhất (UTC).</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:15:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="27" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm xóa mềm; NULL khi bản ghi còn hiệu lực. Không bao giờ xóa hẳn.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Kiểu enum</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Giá trị cho phép</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="27" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>telematicstatus</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>ACTIVE, INACTIVE, MAINTENANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ mục (index)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Các cột</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Duy nhất</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>ix_telematics_status</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="27" customHeight="1">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>ix_telematics_telematic_serial</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>telematic_serial</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>ix_telematics_vehicle_id</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>không</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="27" customHeight="1">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>uq_telematics_active_vehicle</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>vehicle_id</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>WHERE deleted_at IS NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Được tham chiếu bởi bảng</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Cột</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>vehicle_telemetry</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>telematic_id</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:H11"/>
+  <autoFilter ref="A6:H16"/>
   <hyperlinks>
     <hyperlink ref="A2" location="'Tổng quan'!A1"/>
-    <hyperlink ref="F8" location="'customer_accounts'!A1"/>
+    <hyperlink ref="F9" location="'vehicles'!A1"/>
+    <hyperlink ref="B28" location="'vehicle_telemetry'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>